<commit_message>
M03: automate overdue rent + interest accrual on deposit ledger
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/requirements/M03.xlsx
+++ b/requirements/M03.xlsx
@@ -549,7 +549,7 @@
           <t>SRS Reference</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="0" t="inlineStr">
         <is>
           <t>Developer Remarks</t>
         </is>
@@ -679,7 +679,7 @@
           <t>§6.1, FR-RENT-001, FR-RENT-002, BR-RENT-01 to BR-RENT-06, UC-RENT-01</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" s="0" t="inlineStr">
         <is>
           <t>Implemented: monthly draft rent invoice cron (server/cron-rent-invoices.ts) + secured trigger /api/cron/rent-invoice-generation + optional scheduler (server/index.ts).</t>
         </is>
@@ -688,7 +688,7 @@
     <row r="3" ht="79.5" customHeight="1" s="8">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Partially Implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -807,9 +807,9 @@
           <t>§6.1, FR-RENT-007, BR-RENT-15 to BR-RENT-22</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Partially implemented: simple interest calculator exists (server/rent-interest.ts) and dishonour hint shows computed interest; full overdue accrual posting not yet automated.</t>
+      <c r="T3" s="0" t="inlineStr">
+        <is>
+          <t>Implemented: daily job marks past-due unpaid Approved invoices Overdue; posts incremental simple interest to rent_deposit_ledger (entryType Interest). Cron: POST /api/cron/m03-rent-arrears-interest (x-cron-secret) or CRON_M03_RENT_ARREARS=true (00:30 UTC). Rate: system_config rent_arrears_interest_percent_per_annum; principal capped by rent+non-GST vs outstanding.</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
           <t>§6.1, FR-RENT-003, BR-RENT-07, BR-RENT-08, §18 Item 8</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T4" s="0" t="inlineStr">
         <is>
           <t>Implemented: GSTR-1 export endpoint /api/ioms/rent/gstr1 backed by server/rent-gstr1.ts; UI export button in Rent invoices page.</t>
         </is>
@@ -1044,7 +1044,7 @@
           <t>§6.1, FR-RENT-004, BR-RENT-09, BR-RENT-10</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T5" s="0" t="inlineStr">
         <is>
           <t>Implemented: invoice Cancelled status (server/workflow.ts) + credit notes CRUD (server/routes-rent-ioms.ts) + UI (client/src/pages/rent/IomsCreditNotes.tsx).</t>
         </is>
@@ -1162,7 +1162,7 @@
           <t>§6.1, FR-RENT-005, BR-RENT-11, BR-RENT-12</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T6" s="0" t="inlineStr">
         <is>
           <t>Implemented: TDS computation (server/rent-invoice-tds.ts) wired into invoice create/update; receipt carries tdsAmount.</t>
         </is>
@@ -1284,7 +1284,7 @@
           <t>§6.1, FR-RENT-006, BR-RENT-13, BR-RENT-14</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T7" s="0" t="inlineStr">
         <is>
           <t>Implemented (basic): outstanding dues available via M-02 Outstanding dues UI and rent invoice list filters; can extend to ageing buckets if required.</t>
         </is>
@@ -1416,7 +1416,7 @@
           <t>§5.5.3, FR-CHG-001, FR-CHG-002, FR-CHG-003, BR-CHG-01 to BR-CHG-10</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T8" s="0" t="inlineStr">
         <is>
           <t>Implemented (Phase-1): non-GST charge line support stored on rent_invoices.non_gst_charges_json (migration 030) and create-invoice UI supports one optional line; totals include it.</t>
         </is>
@@ -1538,7 +1538,7 @@
           <t>§6.1, FR-RENT-001, BR-RENT-03, BR-RENT-04, E-RENT-001 to E-RENT-003, SCR-RENT-01</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="T9" s="0" t="inlineStr">
         <is>
           <t>Implemented: manual trigger available via /api/cron/rent-invoice-generation (CRON_SECRET protected).</t>
         </is>

</xml_diff>